<commit_message>
Regenerate outputs with corrected GS1 check digit algorithm
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/2026-02-04/quality_by_entity.xlsx
+++ b/outputs/2026-02-04/quality_by_entity.xlsx
@@ -490,10 +490,10 @@
         <v>32054</v>
       </c>
       <c r="C2" t="n">
-        <v>8173</v>
+        <v>24045</v>
       </c>
       <c r="D2" t="n">
-        <v>16433</v>
+        <v>561</v>
       </c>
       <c r="E2" t="n">
         <v>5726</v>
@@ -502,13 +502,13 @@
         <v>1722</v>
       </c>
       <c r="G2" t="n">
-        <v>25.5</v>
+        <v>75.01000000000001</v>
       </c>
       <c r="H2" t="n">
         <v>5</v>
       </c>
       <c r="I2" t="n">
-        <v>3973</v>
+        <v>19845</v>
       </c>
       <c r="J2" t="n">
         <v>4195</v>
@@ -524,10 +524,10 @@
         <v>5840</v>
       </c>
       <c r="C3" t="n">
-        <v>1146</v>
+        <v>1769</v>
       </c>
       <c r="D3" t="n">
-        <v>1246</v>
+        <v>623</v>
       </c>
       <c r="E3" t="n">
         <v>2043</v>
@@ -536,13 +536,13 @@
         <v>1405</v>
       </c>
       <c r="G3" t="n">
-        <v>19.62</v>
+        <v>30.29</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>254</v>
+        <v>877</v>
       </c>
       <c r="J3" t="n">
         <v>892</v>
@@ -558,10 +558,10 @@
         <v>703</v>
       </c>
       <c r="C4" t="n">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>256</v>
@@ -570,13 +570,13 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>63.44</v>
+        <v>63.58</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>446</v>
@@ -592,10 +592,10 @@
         <v>4563</v>
       </c>
       <c r="C5" t="n">
-        <v>290</v>
+        <v>646</v>
       </c>
       <c r="D5" t="n">
-        <v>740</v>
+        <v>384</v>
       </c>
       <c r="E5" t="n">
         <v>3105</v>
@@ -604,13 +604,13 @@
         <v>428</v>
       </c>
       <c r="G5" t="n">
-        <v>6.36</v>
+        <v>14.16</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>92</v>
+        <v>448</v>
       </c>
       <c r="J5" t="n">
         <v>198</v>
@@ -626,10 +626,10 @@
         <v>2257</v>
       </c>
       <c r="C6" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>2119</v>
@@ -638,13 +638,13 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>6.07</v>
+        <v>6.11</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
         <v>136</v>
@@ -660,10 +660,10 @@
         <v>4091</v>
       </c>
       <c r="C7" t="n">
-        <v>695</v>
+        <v>2322</v>
       </c>
       <c r="D7" t="n">
-        <v>1776</v>
+        <v>149</v>
       </c>
       <c r="E7" t="n">
         <v>720</v>
@@ -672,13 +672,13 @@
         <v>900</v>
       </c>
       <c r="G7" t="n">
-        <v>16.99</v>
+        <v>56.76</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>407</v>
+        <v>2034</v>
       </c>
       <c r="J7" t="n">
         <v>286</v>
@@ -728,10 +728,10 @@
         <v>2987</v>
       </c>
       <c r="C9" t="n">
-        <v>658</v>
+        <v>2159</v>
       </c>
       <c r="D9" t="n">
-        <v>1524</v>
+        <v>23</v>
       </c>
       <c r="E9" t="n">
         <v>805</v>
@@ -740,13 +740,13 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>22.03</v>
+        <v>72.28</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>395</v>
+        <v>1896</v>
       </c>
       <c r="J9" t="n">
         <v>263</v>
@@ -762,10 +762,10 @@
         <v>42743</v>
       </c>
       <c r="C10" t="n">
-        <v>25669</v>
+        <v>27113</v>
       </c>
       <c r="D10" t="n">
-        <v>1445</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>15629</v>
@@ -774,13 +774,13 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>60.05</v>
+        <v>63.43</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>363</v>
+        <v>1807</v>
       </c>
       <c r="J10" t="n">
         <v>25306</v>
@@ -796,10 +796,10 @@
         <v>1768</v>
       </c>
       <c r="C11" t="n">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>1222</v>
@@ -808,13 +808,13 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>30.83</v>
+        <v>30.88</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
         <v>545</v>
@@ -864,10 +864,10 @@
         <v>10461</v>
       </c>
       <c r="C13" t="n">
-        <v>4651</v>
+        <v>9847</v>
       </c>
       <c r="D13" t="n">
-        <v>5207</v>
+        <v>11</v>
       </c>
       <c r="E13" t="n">
         <v>599</v>
@@ -876,13 +876,13 @@
         <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>44.46</v>
+        <v>94.13</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1362</v>
+        <v>6558</v>
       </c>
       <c r="J13" t="n">
         <v>3289</v>
@@ -898,10 +898,10 @@
         <v>20675</v>
       </c>
       <c r="C14" t="n">
-        <v>4408</v>
+        <v>11815</v>
       </c>
       <c r="D14" t="n">
-        <v>7716</v>
+        <v>309</v>
       </c>
       <c r="E14" t="n">
         <v>7064</v>
@@ -910,13 +910,13 @@
         <v>1487</v>
       </c>
       <c r="G14" t="n">
-        <v>21.32</v>
+        <v>57.15</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>1849</v>
+        <v>9256</v>
       </c>
       <c r="J14" t="n">
         <v>2558</v>
@@ -932,10 +932,10 @@
         <v>15330</v>
       </c>
       <c r="C15" t="n">
-        <v>3413</v>
+        <v>10185</v>
       </c>
       <c r="D15" t="n">
-        <v>7030</v>
+        <v>258</v>
       </c>
       <c r="E15" t="n">
         <v>4835</v>
@@ -944,13 +944,13 @@
         <v>52</v>
       </c>
       <c r="G15" t="n">
-        <v>22.26</v>
+        <v>66.44</v>
       </c>
       <c r="H15" t="n">
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>1693</v>
+        <v>8465</v>
       </c>
       <c r="J15" t="n">
         <v>1719</v>

</xml_diff>